<commit_message>
fix(restaurant-checklists-en): ronda 1 de la revisión adversarial — 4 MAYOR + 15 menor aplicados
Cuadre de caja con la Z del POS (+ tax, sin propinas), nómina según la frecuencia estatal, enfriamiento
FDA 3-501.14 y tiras de sanitizante en sus filas, turnos AM/Mid/PM, Super Bowl, Labor Day, FLSA estatal,
filtrado de aceite según fabricante. Sin cambios de estructura. G1-G8 verdes, autotest 16/16, censo 0.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/restaurant-checklist-templates/01-opening-closing-checklists-kitchen-foh-bar.xlsx
+++ b/astro-site/public/dl/restaurant-checklist-templates/01-opening-closing-checklists-kitchen-foh-bar.xlsx
@@ -833,7 +833,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="B10" s="41" t="inlineStr">
         <is>
-          <t>▸ File the signed sheets — they prove operational control</t>
+          <t>▸ File the signed sheets — they prove the work was done, and who did it</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
     <row r="35" ht="31" customHeight="1">
       <c r="B35" s="41" t="inlineStr">
         <is>
-          <t>▸ 08-restaurant-opening-closing-checklist.xlsx — checklist for the WHOLE RESTAURANT: it is the FRAME of the day.</t>
+          <t>▸ 08-restaurant-opening-closing-checklist.xlsx — checklist for the WHOLE RESTAURANT: it is the BACKBONE of the day.</t>
         </is>
       </c>
     </row>
@@ -969,7 +969,7 @@
     <row r="39" ht="32" customHeight="1">
       <c r="B39" s="41" t="inlineStr">
         <is>
-          <t>▸ You are in 01-opening-closing-checklists-kitchen-foh-bar.xlsx: it is one MORE layer, not a repeat — the frame of the day is in 08-restaurant-opening-closing-checklist.xlsx.</t>
+          <t>▸ You are in 01-opening-closing-checklists-kitchen-foh-bar.xlsx: it is one MORE layer, not a repeat — the backbone of the day is in 08-restaurant-opening-closing-checklist.xlsx.</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Date: ___/___/______    Shift: ☐ AM  ☐ PM  ☐ Overnight    Shift manager: _________________________</t>
+          <t>Date: ___/___/______    Shift: ☐ AM  ☐ Mid  ☐ PM    Shift manager: _________________________</t>
         </is>
       </c>
     </row>
@@ -1212,7 +1212,7 @@
       </c>
       <c r="B10" s="46" t="inlineStr">
         <is>
-          <t>Report vomiting, diarrhea, jaundice or sore throat with fever to the person in charge; no food handling</t>
+          <t>Check no one has vomiting, diarrhea, jaundice, sore throat with fever or an infected cut; if so, no food handling (FDA 2-201.11)</t>
         </is>
       </c>
       <c r="C10" s="47" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="B17" s="46" t="inlineStr">
         <is>
-          <t>Turn on the dishwasher and check chemical levels</t>
+          <t>Turn on the dish machine and check chemical levels (chemical sanitizing: test strips, ppm on the label)</t>
         </is>
       </c>
       <c r="C17" s="47" t="inlineStr">
@@ -2174,7 +2174,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Date: ___/___/______    Shift: ☐ AM  ☐ PM  ☐ Overnight    Shift manager: _________________________</t>
+          <t>Date: ___/___/______    Shift: ☐ AM  ☐ Mid  ☐ PM    Shift manager: _________________________</t>
         </is>
       </c>
     </row>
@@ -2934,7 +2934,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Date: ___/___/______    Shift: ☐ AM  ☐ PM  ☐ Overnight    Shift manager: _________________________</t>
+          <t>Date: ___/___/______    Shift: ☐ AM  ☐ Mid  ☐ PM    Shift manager: _________________________</t>
         </is>
       </c>
     </row>
@@ -3617,7 +3617,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Date: ___/___/______    Shift: ☐ AM  ☐ PM  ☐ Overnight    Shift manager: _________________________</t>
+          <t>Date: ___/___/______    Shift: ☐ AM  ☐ Mid  ☐ PM    Shift manager: _________________________</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3888,7 @@
       </c>
       <c r="B15" s="46" t="inlineStr">
         <is>
-          <t>Clean and sanitize work surfaces</t>
+          <t>Clean and sanitize work surfaces; test the sanitizer with test strips (ppm on the label)</t>
         </is>
       </c>
       <c r="C15" s="47" t="inlineStr">
@@ -4566,7 +4566,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Date: ___/___/______    Shift: ☐ AM  ☐ PM  ☐ Overnight    Shift manager: _________________________</t>
+          <t>Date: ___/___/______    Shift: ☐ AM  ☐ Mid  ☐ PM    Shift manager: _________________________</t>
         </is>
       </c>
     </row>
@@ -5110,7 +5110,7 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Date: ___/___/______    Shift: ☐ AM  ☐ PM  ☐ Overnight    Shift manager: _________________________</t>
+          <t>Date: ___/___/______    Shift: ☐ AM  ☐ Mid  ☐ PM    Shift manager: _________________________</t>
         </is>
       </c>
     </row>

</xml_diff>